<commit_message>
Add fix_detail_rows.py; hide repeated labels and clear Optimal Count on detail rows
- White font on cols A–E of every detail row so repeated variant text is
  visually invisible while values remain for formula references
- Clear Optimal Count (col I) on detail rows so it only appears on each
  variant's summary row
- F/G/H/J formula placement on summary rows verified unchanged

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inventory_master.xlsx
+++ b/inventory_master.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,6 +37,11 @@
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -191,7 +196,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -241,6 +246,18 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -853,27 +870,27 @@
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>Valencia</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>32" x 80"</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="20" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="20" t="inlineStr">
         <is>
           <t>Left Inswing</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="20" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -881,9 +898,7 @@
       <c r="F4" s="10" t="n"/>
       <c r="G4" s="10" t="n"/>
       <c r="H4" s="10" t="n"/>
-      <c r="I4" s="10" t="n">
-        <v>6</v>
-      </c>
+      <c r="I4" s="10" t="n"/>
       <c r="J4" s="10" t="n"/>
       <c r="K4" s="10" t="inlineStr">
         <is>
@@ -897,27 +912,27 @@
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>Valencia</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="20" t="inlineStr">
         <is>
           <t>32" x 80"</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="20" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="20" t="inlineStr">
         <is>
           <t>Left Inswing</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="20" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -925,9 +940,7 @@
       <c r="F5" s="10" t="n"/>
       <c r="G5" s="10" t="n"/>
       <c r="H5" s="10" t="n"/>
-      <c r="I5" s="10" t="n">
-        <v>6</v>
-      </c>
+      <c r="I5" s="10" t="n"/>
       <c r="J5" s="10" t="n"/>
       <c r="K5" s="10" t="inlineStr">
         <is>
@@ -941,27 +954,27 @@
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t>Valencia</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="20" t="inlineStr">
         <is>
           <t>32" x 80"</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="20" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="20" t="inlineStr">
         <is>
           <t>Left Inswing</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="20" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -969,9 +982,7 @@
       <c r="F6" s="10" t="n"/>
       <c r="G6" s="10" t="n"/>
       <c r="H6" s="10" t="n"/>
-      <c r="I6" s="10" t="n">
-        <v>6</v>
-      </c>
+      <c r="I6" s="10" t="n"/>
       <c r="J6" s="10" t="n"/>
       <c r="K6" s="10" t="inlineStr">
         <is>
@@ -1055,27 +1066,27 @@
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>Valencia</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="20" t="inlineStr">
         <is>
           <t>36" x 80"</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="20" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="20" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -1083,9 +1094,7 @@
       <c r="F9" s="10" t="n"/>
       <c r="G9" s="10" t="n"/>
       <c r="H9" s="10" t="n"/>
-      <c r="I9" s="10" t="n">
-        <v>8</v>
-      </c>
+      <c r="I9" s="10" t="n"/>
       <c r="J9" s="10" t="n"/>
       <c r="K9" s="10" t="inlineStr">
         <is>
@@ -1099,27 +1108,27 @@
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>Valencia</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="20" t="inlineStr">
         <is>
           <t>36" x 80"</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="20" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="E10" s="20" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -1127,9 +1136,7 @@
       <c r="F10" s="10" t="n"/>
       <c r="G10" s="10" t="n"/>
       <c r="H10" s="10" t="n"/>
-      <c r="I10" s="10" t="n">
-        <v>8</v>
-      </c>
+      <c r="I10" s="10" t="n"/>
       <c r="J10" s="10" t="n"/>
       <c r="K10" s="10" t="inlineStr">
         <is>
@@ -1143,27 +1150,27 @@
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>Valencia</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr">
         <is>
           <t>36" x 80"</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E11" s="20" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -1171,9 +1178,7 @@
       <c r="F11" s="10" t="n"/>
       <c r="G11" s="10" t="n"/>
       <c r="H11" s="10" t="n"/>
-      <c r="I11" s="10" t="n">
-        <v>8</v>
-      </c>
+      <c r="I11" s="10" t="n"/>
       <c r="J11" s="10" t="n"/>
       <c r="K11" s="10" t="inlineStr">
         <is>
@@ -1187,27 +1192,27 @@
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>Valencia</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>36" x 80"</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="20" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E12" s="20" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -1215,9 +1220,7 @@
       <c r="F12" s="10" t="n"/>
       <c r="G12" s="10" t="n"/>
       <c r="H12" s="10" t="n"/>
-      <c r="I12" s="10" t="n">
-        <v>8</v>
-      </c>
+      <c r="I12" s="10" t="n"/>
       <c r="J12" s="10" t="n"/>
       <c r="K12" s="10" t="inlineStr">
         <is>
@@ -1231,27 +1234,27 @@
       </c>
     </row>
     <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>Valencia</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="20" t="inlineStr">
         <is>
           <t>36" x 80"</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C13" s="20" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D13" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="E13" s="20" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -1259,9 +1262,7 @@
       <c r="F13" s="10" t="n"/>
       <c r="G13" s="10" t="n"/>
       <c r="H13" s="10" t="n"/>
-      <c r="I13" s="10" t="n">
-        <v>8</v>
-      </c>
+      <c r="I13" s="10" t="n"/>
       <c r="J13" s="10" t="n"/>
       <c r="K13" s="10" t="inlineStr">
         <is>
@@ -1275,27 +1276,27 @@
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>Valencia</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="20" t="inlineStr">
         <is>
           <t>36" x 80"</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="20" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D14" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E14" s="20" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -1303,9 +1304,7 @@
       <c r="F14" s="10" t="n"/>
       <c r="G14" s="10" t="n"/>
       <c r="H14" s="10" t="n"/>
-      <c r="I14" s="10" t="n">
-        <v>8</v>
-      </c>
+      <c r="I14" s="10" t="n"/>
       <c r="J14" s="10" t="n"/>
       <c r="K14" s="10" t="inlineStr">
         <is>
@@ -1389,27 +1388,27 @@
       </c>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="12" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>Valencia</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="22" t="inlineStr">
         <is>
           <t>36" x 96"</t>
         </is>
       </c>
-      <c r="C17" s="13" t="inlineStr">
+      <c r="C17" s="22" t="inlineStr">
         <is>
           <t>Oil-Rubbed Bronze</t>
         </is>
       </c>
-      <c r="D17" s="13" t="inlineStr">
+      <c r="D17" s="22" t="inlineStr">
         <is>
           <t>Right Outswing</t>
         </is>
       </c>
-      <c r="E17" s="13" t="inlineStr">
+      <c r="E17" s="22" t="inlineStr">
         <is>
           <t>Frosted</t>
         </is>
@@ -1417,9 +1416,7 @@
       <c r="F17" s="14" t="n"/>
       <c r="G17" s="14" t="n"/>
       <c r="H17" s="14" t="n"/>
-      <c r="I17" s="14" t="n">
-        <v>6</v>
-      </c>
+      <c r="I17" s="14" t="n"/>
       <c r="J17" s="14" t="n"/>
       <c r="K17" s="14" t="inlineStr">
         <is>
@@ -1517,27 +1514,27 @@
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="19" t="inlineStr">
         <is>
           <t>Sevilla</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="20" t="inlineStr">
         <is>
           <t>32" x 80"</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C21" s="20" t="inlineStr">
         <is>
           <t>Brushed Nickel</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D21" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E21" s="9" t="inlineStr">
+      <c r="E21" s="20" t="inlineStr">
         <is>
           <t>Rain</t>
         </is>
@@ -1545,9 +1542,7 @@
       <c r="F21" s="10" t="n"/>
       <c r="G21" s="10" t="n"/>
       <c r="H21" s="10" t="n"/>
-      <c r="I21" s="10" t="n">
-        <v>7</v>
-      </c>
+      <c r="I21" s="10" t="n"/>
       <c r="J21" s="10" t="n"/>
       <c r="K21" s="10" t="inlineStr">
         <is>
@@ -1561,27 +1556,27 @@
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A22" s="19" t="inlineStr">
         <is>
           <t>Sevilla</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="20" t="inlineStr">
         <is>
           <t>32" x 80"</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
+      <c r="C22" s="20" t="inlineStr">
         <is>
           <t>Brushed Nickel</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="D22" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E22" s="9" t="inlineStr">
+      <c r="E22" s="20" t="inlineStr">
         <is>
           <t>Rain</t>
         </is>
@@ -1589,9 +1584,7 @@
       <c r="F22" s="10" t="n"/>
       <c r="G22" s="10" t="n"/>
       <c r="H22" s="10" t="n"/>
-      <c r="I22" s="10" t="n">
-        <v>7</v>
-      </c>
+      <c r="I22" s="10" t="n"/>
       <c r="J22" s="10" t="n"/>
       <c r="K22" s="10" t="inlineStr">
         <is>
@@ -1605,27 +1598,27 @@
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>Sevilla</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="20" t="inlineStr">
         <is>
           <t>32" x 80"</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
+      <c r="C23" s="20" t="inlineStr">
         <is>
           <t>Brushed Nickel</t>
         </is>
       </c>
-      <c r="D23" s="9" t="inlineStr">
+      <c r="D23" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E23" s="9" t="inlineStr">
+      <c r="E23" s="20" t="inlineStr">
         <is>
           <t>Rain</t>
         </is>
@@ -1633,9 +1626,7 @@
       <c r="F23" s="10" t="n"/>
       <c r="G23" s="10" t="n"/>
       <c r="H23" s="10" t="n"/>
-      <c r="I23" s="10" t="n">
-        <v>7</v>
-      </c>
+      <c r="I23" s="10" t="n"/>
       <c r="J23" s="10" t="n"/>
       <c r="K23" s="10" t="inlineStr">
         <is>
@@ -1649,27 +1640,27 @@
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="8" t="inlineStr">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t>Sevilla</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="20" t="inlineStr">
         <is>
           <t>32" x 80"</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
+      <c r="C24" s="20" t="inlineStr">
         <is>
           <t>Brushed Nickel</t>
         </is>
       </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="D24" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E24" s="9" t="inlineStr">
+      <c r="E24" s="20" t="inlineStr">
         <is>
           <t>Rain</t>
         </is>
@@ -1677,9 +1668,7 @@
       <c r="F24" s="10" t="n"/>
       <c r="G24" s="10" t="n"/>
       <c r="H24" s="10" t="n"/>
-      <c r="I24" s="10" t="n">
-        <v>7</v>
-      </c>
+      <c r="I24" s="10" t="n"/>
       <c r="J24" s="10" t="n"/>
       <c r="K24" s="10" t="inlineStr">
         <is>
@@ -1763,27 +1752,27 @@
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="8" t="inlineStr">
+      <c r="A27" s="19" t="inlineStr">
         <is>
           <t>Sevilla</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B27" s="20" t="inlineStr">
         <is>
           <t>36" x 80"</t>
         </is>
       </c>
-      <c r="C27" s="9" t="inlineStr">
+      <c r="C27" s="20" t="inlineStr">
         <is>
           <t>Satin White</t>
         </is>
       </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="D27" s="20" t="inlineStr">
         <is>
           <t>Left Inswing</t>
         </is>
       </c>
-      <c r="E27" s="9" t="inlineStr">
+      <c r="E27" s="20" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -1791,9 +1780,7 @@
       <c r="F27" s="10" t="n"/>
       <c r="G27" s="10" t="n"/>
       <c r="H27" s="10" t="n"/>
-      <c r="I27" s="10" t="n">
-        <v>8</v>
-      </c>
+      <c r="I27" s="10" t="n"/>
       <c r="J27" s="10" t="n"/>
       <c r="K27" s="10" t="inlineStr">
         <is>
@@ -1807,27 +1794,27 @@
       </c>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="12" t="inlineStr">
+      <c r="A28" s="21" t="inlineStr">
         <is>
           <t>Sevilla</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="B28" s="22" t="inlineStr">
         <is>
           <t>36" x 80"</t>
         </is>
       </c>
-      <c r="C28" s="13" t="inlineStr">
+      <c r="C28" s="22" t="inlineStr">
         <is>
           <t>Satin White</t>
         </is>
       </c>
-      <c r="D28" s="13" t="inlineStr">
+      <c r="D28" s="22" t="inlineStr">
         <is>
           <t>Left Inswing</t>
         </is>
       </c>
-      <c r="E28" s="13" t="inlineStr">
+      <c r="E28" s="22" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -1835,9 +1822,7 @@
       <c r="F28" s="14" t="n"/>
       <c r="G28" s="14" t="n"/>
       <c r="H28" s="14" t="n"/>
-      <c r="I28" s="14" t="n">
-        <v>8</v>
-      </c>
+      <c r="I28" s="14" t="n"/>
       <c r="J28" s="14" t="n"/>
       <c r="K28" s="14" t="inlineStr">
         <is>
@@ -1935,27 +1920,27 @@
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="A32" s="19" t="inlineStr">
         <is>
           <t>Cordova</t>
         </is>
       </c>
-      <c r="B32" s="9" t="inlineStr">
+      <c r="B32" s="20" t="inlineStr">
         <is>
           <t>32" x 80"</t>
         </is>
       </c>
-      <c r="C32" s="9" t="inlineStr">
+      <c r="C32" s="20" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D32" s="9" t="inlineStr">
+      <c r="D32" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E32" s="9" t="inlineStr">
+      <c r="E32" s="20" t="inlineStr">
         <is>
           <t>Frosted</t>
         </is>
@@ -1963,9 +1948,7 @@
       <c r="F32" s="10" t="n"/>
       <c r="G32" s="10" t="n"/>
       <c r="H32" s="10" t="n"/>
-      <c r="I32" s="10" t="n">
-        <v>7</v>
-      </c>
+      <c r="I32" s="10" t="n"/>
       <c r="J32" s="10" t="n"/>
       <c r="K32" s="10" t="inlineStr">
         <is>
@@ -1979,27 +1962,27 @@
       </c>
     </row>
     <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="A33" s="19" t="inlineStr">
         <is>
           <t>Cordova</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B33" s="20" t="inlineStr">
         <is>
           <t>32" x 80"</t>
         </is>
       </c>
-      <c r="C33" s="9" t="inlineStr">
+      <c r="C33" s="20" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D33" s="9" t="inlineStr">
+      <c r="D33" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E33" s="9" t="inlineStr">
+      <c r="E33" s="20" t="inlineStr">
         <is>
           <t>Frosted</t>
         </is>
@@ -2007,9 +1990,7 @@
       <c r="F33" s="10" t="n"/>
       <c r="G33" s="10" t="n"/>
       <c r="H33" s="10" t="n"/>
-      <c r="I33" s="10" t="n">
-        <v>7</v>
-      </c>
+      <c r="I33" s="10" t="n"/>
       <c r="J33" s="10" t="n"/>
       <c r="K33" s="10" t="inlineStr">
         <is>
@@ -2023,27 +2004,27 @@
       </c>
     </row>
     <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="8" t="inlineStr">
+      <c r="A34" s="19" t="inlineStr">
         <is>
           <t>Cordova</t>
         </is>
       </c>
-      <c r="B34" s="9" t="inlineStr">
+      <c r="B34" s="20" t="inlineStr">
         <is>
           <t>32" x 80"</t>
         </is>
       </c>
-      <c r="C34" s="9" t="inlineStr">
+      <c r="C34" s="20" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D34" s="9" t="inlineStr">
+      <c r="D34" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E34" s="9" t="inlineStr">
+      <c r="E34" s="20" t="inlineStr">
         <is>
           <t>Frosted</t>
         </is>
@@ -2051,9 +2032,7 @@
       <c r="F34" s="10" t="n"/>
       <c r="G34" s="10" t="n"/>
       <c r="H34" s="10" t="n"/>
-      <c r="I34" s="10" t="n">
-        <v>7</v>
-      </c>
+      <c r="I34" s="10" t="n"/>
       <c r="J34" s="10" t="n"/>
       <c r="K34" s="10" t="inlineStr">
         <is>
@@ -2067,27 +2046,27 @@
       </c>
     </row>
     <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="8" t="inlineStr">
+      <c r="A35" s="19" t="inlineStr">
         <is>
           <t>Cordova</t>
         </is>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B35" s="20" t="inlineStr">
         <is>
           <t>32" x 80"</t>
         </is>
       </c>
-      <c r="C35" s="9" t="inlineStr">
+      <c r="C35" s="20" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="D35" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E35" s="9" t="inlineStr">
+      <c r="E35" s="20" t="inlineStr">
         <is>
           <t>Frosted</t>
         </is>
@@ -2095,9 +2074,7 @@
       <c r="F35" s="10" t="n"/>
       <c r="G35" s="10" t="n"/>
       <c r="H35" s="10" t="n"/>
-      <c r="I35" s="10" t="n">
-        <v>7</v>
-      </c>
+      <c r="I35" s="10" t="n"/>
       <c r="J35" s="10" t="n"/>
       <c r="K35" s="10" t="inlineStr">
         <is>
@@ -2111,27 +2088,27 @@
       </c>
     </row>
     <row r="36" ht="16" customHeight="1">
-      <c r="A36" s="8" t="inlineStr">
+      <c r="A36" s="19" t="inlineStr">
         <is>
           <t>Cordova</t>
         </is>
       </c>
-      <c r="B36" s="9" t="inlineStr">
+      <c r="B36" s="20" t="inlineStr">
         <is>
           <t>32" x 80"</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
+      <c r="C36" s="20" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D36" s="9" t="inlineStr">
+      <c r="D36" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E36" s="9" t="inlineStr">
+      <c r="E36" s="20" t="inlineStr">
         <is>
           <t>Frosted</t>
         </is>
@@ -2139,9 +2116,7 @@
       <c r="F36" s="10" t="n"/>
       <c r="G36" s="10" t="n"/>
       <c r="H36" s="10" t="n"/>
-      <c r="I36" s="10" t="n">
-        <v>7</v>
-      </c>
+      <c r="I36" s="10" t="n"/>
       <c r="J36" s="10" t="n"/>
       <c r="K36" s="10" t="inlineStr">
         <is>
@@ -2225,27 +2200,27 @@
       </c>
     </row>
     <row r="39" ht="16" customHeight="1">
-      <c r="A39" s="8" t="inlineStr">
+      <c r="A39" s="19" t="inlineStr">
         <is>
           <t>Cordova</t>
         </is>
       </c>
-      <c r="B39" s="9" t="inlineStr">
+      <c r="B39" s="20" t="inlineStr">
         <is>
           <t>36" x 80"</t>
         </is>
       </c>
-      <c r="C39" s="9" t="inlineStr">
+      <c r="C39" s="20" t="inlineStr">
         <is>
           <t>Oil-Rubbed Bronze</t>
         </is>
       </c>
-      <c r="D39" s="9" t="inlineStr">
+      <c r="D39" s="20" t="inlineStr">
         <is>
           <t>Left Inswing</t>
         </is>
       </c>
-      <c r="E39" s="9" t="inlineStr">
+      <c r="E39" s="20" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -2253,9 +2228,7 @@
       <c r="F39" s="10" t="n"/>
       <c r="G39" s="10" t="n"/>
       <c r="H39" s="10" t="n"/>
-      <c r="I39" s="10" t="n">
-        <v>9</v>
-      </c>
+      <c r="I39" s="10" t="n"/>
       <c r="J39" s="10" t="n"/>
       <c r="K39" s="10" t="inlineStr">
         <is>
@@ -2269,27 +2242,27 @@
       </c>
     </row>
     <row r="40" ht="16" customHeight="1">
-      <c r="A40" s="8" t="inlineStr">
+      <c r="A40" s="19" t="inlineStr">
         <is>
           <t>Cordova</t>
         </is>
       </c>
-      <c r="B40" s="9" t="inlineStr">
+      <c r="B40" s="20" t="inlineStr">
         <is>
           <t>36" x 80"</t>
         </is>
       </c>
-      <c r="C40" s="9" t="inlineStr">
+      <c r="C40" s="20" t="inlineStr">
         <is>
           <t>Oil-Rubbed Bronze</t>
         </is>
       </c>
-      <c r="D40" s="9" t="inlineStr">
+      <c r="D40" s="20" t="inlineStr">
         <is>
           <t>Left Inswing</t>
         </is>
       </c>
-      <c r="E40" s="9" t="inlineStr">
+      <c r="E40" s="20" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -2297,9 +2270,7 @@
       <c r="F40" s="10" t="n"/>
       <c r="G40" s="10" t="n"/>
       <c r="H40" s="10" t="n"/>
-      <c r="I40" s="10" t="n">
-        <v>9</v>
-      </c>
+      <c r="I40" s="10" t="n"/>
       <c r="J40" s="10" t="n"/>
       <c r="K40" s="10" t="inlineStr">
         <is>
@@ -2467,27 +2438,27 @@
       </c>
     </row>
     <row r="46" ht="16" customHeight="1">
-      <c r="A46" s="8" t="inlineStr">
+      <c r="A46" s="19" t="inlineStr">
         <is>
           <t>Granada</t>
         </is>
       </c>
-      <c r="B46" s="9" t="inlineStr">
+      <c r="B46" s="20" t="inlineStr">
         <is>
           <t>36" x 80"</t>
         </is>
       </c>
-      <c r="C46" s="9" t="inlineStr">
+      <c r="C46" s="20" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D46" s="9" t="inlineStr">
+      <c r="D46" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E46" s="9" t="inlineStr">
+      <c r="E46" s="20" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -2495,9 +2466,7 @@
       <c r="F46" s="10" t="n"/>
       <c r="G46" s="10" t="n"/>
       <c r="H46" s="10" t="n"/>
-      <c r="I46" s="10" t="n">
-        <v>8</v>
-      </c>
+      <c r="I46" s="10" t="n"/>
       <c r="J46" s="10" t="n"/>
       <c r="K46" s="10" t="inlineStr">
         <is>
@@ -2511,27 +2480,27 @@
       </c>
     </row>
     <row r="47" ht="16" customHeight="1">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="A47" s="19" t="inlineStr">
         <is>
           <t>Granada</t>
         </is>
       </c>
-      <c r="B47" s="9" t="inlineStr">
+      <c r="B47" s="20" t="inlineStr">
         <is>
           <t>36" x 80"</t>
         </is>
       </c>
-      <c r="C47" s="9" t="inlineStr">
+      <c r="C47" s="20" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D47" s="9" t="inlineStr">
+      <c r="D47" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E47" s="9" t="inlineStr">
+      <c r="E47" s="20" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -2539,9 +2508,7 @@
       <c r="F47" s="10" t="n"/>
       <c r="G47" s="10" t="n"/>
       <c r="H47" s="10" t="n"/>
-      <c r="I47" s="10" t="n">
-        <v>8</v>
-      </c>
+      <c r="I47" s="10" t="n"/>
       <c r="J47" s="10" t="n"/>
       <c r="K47" s="10" t="inlineStr">
         <is>
@@ -2555,27 +2522,27 @@
       </c>
     </row>
     <row r="48" ht="16" customHeight="1">
-      <c r="A48" s="8" t="inlineStr">
+      <c r="A48" s="19" t="inlineStr">
         <is>
           <t>Granada</t>
         </is>
       </c>
-      <c r="B48" s="9" t="inlineStr">
+      <c r="B48" s="20" t="inlineStr">
         <is>
           <t>36" x 80"</t>
         </is>
       </c>
-      <c r="C48" s="9" t="inlineStr">
+      <c r="C48" s="20" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D48" s="9" t="inlineStr">
+      <c r="D48" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E48" s="9" t="inlineStr">
+      <c r="E48" s="20" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -2583,9 +2550,7 @@
       <c r="F48" s="10" t="n"/>
       <c r="G48" s="10" t="n"/>
       <c r="H48" s="10" t="n"/>
-      <c r="I48" s="10" t="n">
-        <v>8</v>
-      </c>
+      <c r="I48" s="10" t="n"/>
       <c r="J48" s="10" t="n"/>
       <c r="K48" s="10" t="inlineStr">
         <is>
@@ -2599,27 +2564,27 @@
       </c>
     </row>
     <row r="49" ht="16" customHeight="1">
-      <c r="A49" s="8" t="inlineStr">
+      <c r="A49" s="19" t="inlineStr">
         <is>
           <t>Granada</t>
         </is>
       </c>
-      <c r="B49" s="9" t="inlineStr">
+      <c r="B49" s="20" t="inlineStr">
         <is>
           <t>36" x 80"</t>
         </is>
       </c>
-      <c r="C49" s="9" t="inlineStr">
+      <c r="C49" s="20" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D49" s="9" t="inlineStr">
+      <c r="D49" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E49" s="9" t="inlineStr">
+      <c r="E49" s="20" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -2627,9 +2592,7 @@
       <c r="F49" s="10" t="n"/>
       <c r="G49" s="10" t="n"/>
       <c r="H49" s="10" t="n"/>
-      <c r="I49" s="10" t="n">
-        <v>8</v>
-      </c>
+      <c r="I49" s="10" t="n"/>
       <c r="J49" s="10" t="n"/>
       <c r="K49" s="10" t="inlineStr">
         <is>
@@ -2643,27 +2606,27 @@
       </c>
     </row>
     <row r="50" ht="16" customHeight="1">
-      <c r="A50" s="8" t="inlineStr">
+      <c r="A50" s="19" t="inlineStr">
         <is>
           <t>Granada</t>
         </is>
       </c>
-      <c r="B50" s="9" t="inlineStr">
+      <c r="B50" s="20" t="inlineStr">
         <is>
           <t>36" x 80"</t>
         </is>
       </c>
-      <c r="C50" s="9" t="inlineStr">
+      <c r="C50" s="20" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D50" s="9" t="inlineStr">
+      <c r="D50" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E50" s="9" t="inlineStr">
+      <c r="E50" s="20" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -2671,9 +2634,7 @@
       <c r="F50" s="10" t="n"/>
       <c r="G50" s="10" t="n"/>
       <c r="H50" s="10" t="n"/>
-      <c r="I50" s="10" t="n">
-        <v>8</v>
-      </c>
+      <c r="I50" s="10" t="n"/>
       <c r="J50" s="10" t="n"/>
       <c r="K50" s="10" t="inlineStr">
         <is>
@@ -2687,27 +2648,27 @@
       </c>
     </row>
     <row r="51" ht="16" customHeight="1">
-      <c r="A51" s="8" t="inlineStr">
+      <c r="A51" s="19" t="inlineStr">
         <is>
           <t>Granada</t>
         </is>
       </c>
-      <c r="B51" s="9" t="inlineStr">
+      <c r="B51" s="20" t="inlineStr">
         <is>
           <t>36" x 80"</t>
         </is>
       </c>
-      <c r="C51" s="9" t="inlineStr">
+      <c r="C51" s="20" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D51" s="9" t="inlineStr">
+      <c r="D51" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E51" s="9" t="inlineStr">
+      <c r="E51" s="20" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -2715,9 +2676,7 @@
       <c r="F51" s="10" t="n"/>
       <c r="G51" s="10" t="n"/>
       <c r="H51" s="10" t="n"/>
-      <c r="I51" s="10" t="n">
-        <v>8</v>
-      </c>
+      <c r="I51" s="10" t="n"/>
       <c r="J51" s="10" t="n"/>
       <c r="K51" s="10" t="inlineStr">
         <is>
@@ -2731,27 +2690,27 @@
       </c>
     </row>
     <row r="52" ht="16" customHeight="1">
-      <c r="A52" s="8" t="inlineStr">
+      <c r="A52" s="19" t="inlineStr">
         <is>
           <t>Granada</t>
         </is>
       </c>
-      <c r="B52" s="9" t="inlineStr">
+      <c r="B52" s="20" t="inlineStr">
         <is>
           <t>36" x 80"</t>
         </is>
       </c>
-      <c r="C52" s="9" t="inlineStr">
+      <c r="C52" s="20" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D52" s="9" t="inlineStr">
+      <c r="D52" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E52" s="9" t="inlineStr">
+      <c r="E52" s="20" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -2759,9 +2718,7 @@
       <c r="F52" s="10" t="n"/>
       <c r="G52" s="10" t="n"/>
       <c r="H52" s="10" t="n"/>
-      <c r="I52" s="10" t="n">
-        <v>8</v>
-      </c>
+      <c r="I52" s="10" t="n"/>
       <c r="J52" s="10" t="n"/>
       <c r="K52" s="10" t="inlineStr">
         <is>
@@ -2845,27 +2802,27 @@
       </c>
     </row>
     <row r="55" ht="16" customHeight="1">
-      <c r="A55" s="12" t="inlineStr">
+      <c r="A55" s="21" t="inlineStr">
         <is>
           <t>Granada</t>
         </is>
       </c>
-      <c r="B55" s="13" t="inlineStr">
+      <c r="B55" s="22" t="inlineStr">
         <is>
           <t>36" x 96"</t>
         </is>
       </c>
-      <c r="C55" s="13" t="inlineStr">
+      <c r="C55" s="22" t="inlineStr">
         <is>
           <t>Satin White</t>
         </is>
       </c>
-      <c r="D55" s="13" t="inlineStr">
+      <c r="D55" s="22" t="inlineStr">
         <is>
           <t>Left Inswing</t>
         </is>
       </c>
-      <c r="E55" s="13" t="inlineStr">
+      <c r="E55" s="22" t="inlineStr">
         <is>
           <t>Sidelite</t>
         </is>
@@ -2873,9 +2830,7 @@
       <c r="F55" s="14" t="n"/>
       <c r="G55" s="14" t="n"/>
       <c r="H55" s="14" t="n"/>
-      <c r="I55" s="14" t="n">
-        <v>6</v>
-      </c>
+      <c r="I55" s="14" t="n"/>
       <c r="J55" s="14" t="n"/>
       <c r="K55" s="14" t="inlineStr">
         <is>
@@ -2973,27 +2928,27 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="8" t="inlineStr">
+      <c r="A59" s="19" t="inlineStr">
         <is>
           <t>Malaga</t>
         </is>
       </c>
-      <c r="B59" s="9" t="inlineStr">
+      <c r="B59" s="20" t="inlineStr">
         <is>
           <t>32" x 80"</t>
         </is>
       </c>
-      <c r="C59" s="9" t="inlineStr">
+      <c r="C59" s="20" t="inlineStr">
         <is>
           <t>Brushed Nickel</t>
         </is>
       </c>
-      <c r="D59" s="9" t="inlineStr">
+      <c r="D59" s="20" t="inlineStr">
         <is>
           <t>Left Inswing</t>
         </is>
       </c>
-      <c r="E59" s="9" t="inlineStr">
+      <c r="E59" s="20" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -3001,9 +2956,7 @@
       <c r="F59" s="10" t="n"/>
       <c r="G59" s="10" t="n"/>
       <c r="H59" s="10" t="n"/>
-      <c r="I59" s="10" t="n">
-        <v>5</v>
-      </c>
+      <c r="I59" s="10" t="n"/>
       <c r="J59" s="10" t="n"/>
       <c r="K59" s="10" t="inlineStr">
         <is>
@@ -3017,27 +2970,27 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="8" t="inlineStr">
+      <c r="A60" s="19" t="inlineStr">
         <is>
           <t>Malaga</t>
         </is>
       </c>
-      <c r="B60" s="9" t="inlineStr">
+      <c r="B60" s="20" t="inlineStr">
         <is>
           <t>32" x 80"</t>
         </is>
       </c>
-      <c r="C60" s="9" t="inlineStr">
+      <c r="C60" s="20" t="inlineStr">
         <is>
           <t>Brushed Nickel</t>
         </is>
       </c>
-      <c r="D60" s="9" t="inlineStr">
+      <c r="D60" s="20" t="inlineStr">
         <is>
           <t>Left Inswing</t>
         </is>
       </c>
-      <c r="E60" s="9" t="inlineStr">
+      <c r="E60" s="20" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -3045,9 +2998,7 @@
       <c r="F60" s="10" t="n"/>
       <c r="G60" s="10" t="n"/>
       <c r="H60" s="10" t="n"/>
-      <c r="I60" s="10" t="n">
-        <v>5</v>
-      </c>
+      <c r="I60" s="10" t="n"/>
       <c r="J60" s="10" t="n"/>
       <c r="K60" s="10" t="inlineStr">
         <is>
@@ -3061,27 +3012,27 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="12" t="inlineStr">
+      <c r="A61" s="21" t="inlineStr">
         <is>
           <t>Malaga</t>
         </is>
       </c>
-      <c r="B61" s="13" t="inlineStr">
+      <c r="B61" s="22" t="inlineStr">
         <is>
           <t>32" x 80"</t>
         </is>
       </c>
-      <c r="C61" s="13" t="inlineStr">
+      <c r="C61" s="22" t="inlineStr">
         <is>
           <t>Brushed Nickel</t>
         </is>
       </c>
-      <c r="D61" s="13" t="inlineStr">
+      <c r="D61" s="22" t="inlineStr">
         <is>
           <t>Left Inswing</t>
         </is>
       </c>
-      <c r="E61" s="13" t="inlineStr">
+      <c r="E61" s="22" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -3089,9 +3040,7 @@
       <c r="F61" s="14" t="n"/>
       <c r="G61" s="14" t="n"/>
       <c r="H61" s="14" t="n"/>
-      <c r="I61" s="14" t="n">
-        <v>5</v>
-      </c>
+      <c r="I61" s="14" t="n"/>
       <c r="J61" s="14" t="n"/>
       <c r="K61" s="14" t="inlineStr">
         <is>
@@ -3189,27 +3138,27 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="8" t="inlineStr">
+      <c r="A65" s="19" t="inlineStr">
         <is>
           <t>Altea</t>
         </is>
       </c>
-      <c r="B65" s="9" t="inlineStr">
+      <c r="B65" s="20" t="inlineStr">
         <is>
           <t>32" x 80"</t>
         </is>
       </c>
-      <c r="C65" s="9" t="inlineStr">
+      <c r="C65" s="20" t="inlineStr">
         <is>
           <t>Satin White</t>
         </is>
       </c>
-      <c r="D65" s="9" t="inlineStr">
+      <c r="D65" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E65" s="9" t="inlineStr">
+      <c r="E65" s="20" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -3217,9 +3166,7 @@
       <c r="F65" s="10" t="n"/>
       <c r="G65" s="10" t="n"/>
       <c r="H65" s="10" t="n"/>
-      <c r="I65" s="10" t="n">
-        <v>6</v>
-      </c>
+      <c r="I65" s="10" t="n"/>
       <c r="J65" s="10" t="n"/>
       <c r="K65" s="10" t="inlineStr">
         <is>
@@ -3233,27 +3180,27 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="8" t="inlineStr">
+      <c r="A66" s="19" t="inlineStr">
         <is>
           <t>Altea</t>
         </is>
       </c>
-      <c r="B66" s="9" t="inlineStr">
+      <c r="B66" s="20" t="inlineStr">
         <is>
           <t>32" x 80"</t>
         </is>
       </c>
-      <c r="C66" s="9" t="inlineStr">
+      <c r="C66" s="20" t="inlineStr">
         <is>
           <t>Satin White</t>
         </is>
       </c>
-      <c r="D66" s="9" t="inlineStr">
+      <c r="D66" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E66" s="9" t="inlineStr">
+      <c r="E66" s="20" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -3261,9 +3208,7 @@
       <c r="F66" s="10" t="n"/>
       <c r="G66" s="10" t="n"/>
       <c r="H66" s="10" t="n"/>
-      <c r="I66" s="10" t="n">
-        <v>6</v>
-      </c>
+      <c r="I66" s="10" t="n"/>
       <c r="J66" s="10" t="n"/>
       <c r="K66" s="10" t="inlineStr">
         <is>
@@ -3277,27 +3222,27 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="8" t="inlineStr">
+      <c r="A67" s="19" t="inlineStr">
         <is>
           <t>Altea</t>
         </is>
       </c>
-      <c r="B67" s="9" t="inlineStr">
+      <c r="B67" s="20" t="inlineStr">
         <is>
           <t>32" x 80"</t>
         </is>
       </c>
-      <c r="C67" s="9" t="inlineStr">
+      <c r="C67" s="20" t="inlineStr">
         <is>
           <t>Satin White</t>
         </is>
       </c>
-      <c r="D67" s="9" t="inlineStr">
+      <c r="D67" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E67" s="9" t="inlineStr">
+      <c r="E67" s="20" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -3305,9 +3250,7 @@
       <c r="F67" s="10" t="n"/>
       <c r="G67" s="10" t="n"/>
       <c r="H67" s="10" t="n"/>
-      <c r="I67" s="10" t="n">
-        <v>6</v>
-      </c>
+      <c r="I67" s="10" t="n"/>
       <c r="J67" s="10" t="n"/>
       <c r="K67" s="10" t="inlineStr">
         <is>
@@ -3321,27 +3264,27 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="8" t="inlineStr">
+      <c r="A68" s="19" t="inlineStr">
         <is>
           <t>Altea</t>
         </is>
       </c>
-      <c r="B68" s="9" t="inlineStr">
+      <c r="B68" s="20" t="inlineStr">
         <is>
           <t>32" x 80"</t>
         </is>
       </c>
-      <c r="C68" s="9" t="inlineStr">
+      <c r="C68" s="20" t="inlineStr">
         <is>
           <t>Satin White</t>
         </is>
       </c>
-      <c r="D68" s="9" t="inlineStr">
+      <c r="D68" s="20" t="inlineStr">
         <is>
           <t>Right Inswing</t>
         </is>
       </c>
-      <c r="E68" s="9" t="inlineStr">
+      <c r="E68" s="20" t="inlineStr">
         <is>
           <t>Clear</t>
         </is>
@@ -3349,9 +3292,7 @@
       <c r="F68" s="10" t="n"/>
       <c r="G68" s="10" t="n"/>
       <c r="H68" s="10" t="n"/>
-      <c r="I68" s="10" t="n">
-        <v>6</v>
-      </c>
+      <c r="I68" s="10" t="n"/>
       <c r="J68" s="10" t="n"/>
       <c r="K68" s="10" t="inlineStr">
         <is>
@@ -3435,27 +3376,27 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="8" t="inlineStr">
+      <c r="A71" s="19" t="inlineStr">
         <is>
           <t>Altea</t>
         </is>
       </c>
-      <c r="B71" s="9" t="inlineStr">
+      <c r="B71" s="20" t="inlineStr">
         <is>
           <t>36" x 80"</t>
         </is>
       </c>
-      <c r="C71" s="9" t="inlineStr">
+      <c r="C71" s="20" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D71" s="9" t="inlineStr">
+      <c r="D71" s="20" t="inlineStr">
         <is>
           <t>Left Inswing</t>
         </is>
       </c>
-      <c r="E71" s="9" t="inlineStr">
+      <c r="E71" s="20" t="inlineStr">
         <is>
           <t>Rain</t>
         </is>
@@ -3463,9 +3404,7 @@
       <c r="F71" s="10" t="n"/>
       <c r="G71" s="10" t="n"/>
       <c r="H71" s="10" t="n"/>
-      <c r="I71" s="10" t="n">
-        <v>7</v>
-      </c>
+      <c r="I71" s="10" t="n"/>
       <c r="J71" s="10" t="n"/>
       <c r="K71" s="10" t="inlineStr">
         <is>
@@ -3479,27 +3418,27 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="8" t="inlineStr">
+      <c r="A72" s="19" t="inlineStr">
         <is>
           <t>Altea</t>
         </is>
       </c>
-      <c r="B72" s="9" t="inlineStr">
+      <c r="B72" s="20" t="inlineStr">
         <is>
           <t>36" x 80"</t>
         </is>
       </c>
-      <c r="C72" s="9" t="inlineStr">
+      <c r="C72" s="20" t="inlineStr">
         <is>
           <t>Matte Black</t>
         </is>
       </c>
-      <c r="D72" s="9" t="inlineStr">
+      <c r="D72" s="20" t="inlineStr">
         <is>
           <t>Left Inswing</t>
         </is>
       </c>
-      <c r="E72" s="9" t="inlineStr">
+      <c r="E72" s="20" t="inlineStr">
         <is>
           <t>Rain</t>
         </is>
@@ -3507,9 +3446,7 @@
       <c r="F72" s="10" t="n"/>
       <c r="G72" s="10" t="n"/>
       <c r="H72" s="10" t="n"/>
-      <c r="I72" s="10" t="n">
-        <v>7</v>
-      </c>
+      <c r="I72" s="10" t="n"/>
       <c r="J72" s="10" t="n"/>
       <c r="K72" s="10" t="inlineStr">
         <is>

</xml_diff>